<commit_message>
feat: Excel export of requests by template (signature, one-page print, caps surname) + welcome page text
</commit_message>
<xml_diff>
--- a/public/xls/REQUEST.xlsx
+++ b/public/xls/REQUEST.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\sv-progs-assistant\public\xls\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stanislav/Desktop/PROJECTS/sv-progs-assistant/public/xls/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1846FC9-8D0E-427D-8C7C-A66A1AB71A59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A210701-1BEF-E14D-9385-D20D9B99484A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F3EB26A4-3A24-4C34-A589-8AC17AA75156}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15720" xr2:uid="{F3EB26A4-3A24-4C34-A589-8AC17AA75156}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -60,7 +60,7 @@
     <t>Марк Демешко</t>
   </si>
   <si>
-    <t>Начальник виробничої дільниці   №</t>
+    <t>Начальник виробничої дільниці</t>
   </si>
 </sst>
 </file>
@@ -156,32 +156,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -201,9 +196,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office 2013–2022">
   <a:themeElements>
-    <a:clrScheme name="Стандартная">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -241,7 +236,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Стандартная">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -347,7 +342,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Стандартная">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -489,7 +484,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -498,12 +493,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1934A945-5535-436C-86BE-3BB3E2BBBB5B}">
   <dimension ref="A2:N39"/>
-  <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="18" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="16384" width="9.1640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:14" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" ht="20" x14ac:dyDescent="0.2">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -520,7 +515,7 @@
       <c r="L2" s="3"/>
       <c r="M2" s="3"/>
     </row>
-    <row r="3" spans="1:14" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" ht="20" x14ac:dyDescent="0.2">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -537,7 +532,7 @@
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>
     </row>
-    <row r="4" spans="1:14" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" ht="20" x14ac:dyDescent="0.2">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -552,7 +547,7 @@
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
     </row>
-    <row r="5" spans="1:14" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" ht="20" x14ac:dyDescent="0.2">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -569,7 +564,7 @@
       <c r="L5" s="3"/>
       <c r="M5" s="3"/>
     </row>
-    <row r="6" spans="1:14" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" ht="20" x14ac:dyDescent="0.2">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -586,7 +581,7 @@
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
     </row>
-    <row r="7" spans="1:14" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" ht="20" x14ac:dyDescent="0.2">
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
@@ -601,7 +596,7 @@
       <c r="L7" s="3"/>
       <c r="M7" s="3"/>
     </row>
-    <row r="8" spans="1:14" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" ht="20" x14ac:dyDescent="0.2">
       <c r="A8" s="3"/>
       <c r="B8" s="4"/>
       <c r="C8" s="3" t="s">
@@ -618,7 +613,7 @@
       <c r="L8" s="3"/>
       <c r="M8" s="3"/>
     </row>
-    <row r="9" spans="1:14" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" ht="20" x14ac:dyDescent="0.2">
       <c r="A9" s="4"/>
       <c r="B9" s="3" t="s">
         <v>6</v>
@@ -635,445 +630,376 @@
       <c r="L9" s="3"/>
       <c r="M9" s="3"/>
     </row>
-    <row r="11" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>1</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
-      <c r="H11" s="7"/>
-      <c r="I11" s="7"/>
-      <c r="J11" s="7"/>
-      <c r="K11" s="7"/>
-      <c r="L11" s="7"/>
-      <c r="M11" s="12">
-        <v>5</v>
-      </c>
-      <c r="N11" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="M11" s="9">
+        <v>5</v>
+      </c>
+      <c r="N11" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>2</v>
       </c>
-      <c r="B12" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C12" s="7"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
-      <c r="I12" s="7"/>
-      <c r="J12" s="7"/>
-      <c r="K12" s="7"/>
-      <c r="L12" s="7"/>
-      <c r="M12" s="12">
-        <v>5</v>
-      </c>
-      <c r="N12" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D12" s="7"/>
+      <c r="M12" s="9">
+        <v>5</v>
+      </c>
+      <c r="N12" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>3</v>
       </c>
-      <c r="B13" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
-      <c r="I13" s="7"/>
-      <c r="J13" s="7"/>
-      <c r="K13" s="7"/>
-      <c r="L13" s="7"/>
-      <c r="M13" s="12">
-        <v>5</v>
-      </c>
-      <c r="N13" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="M13" s="9">
+        <v>5</v>
+      </c>
+      <c r="N13" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>4</v>
       </c>
-      <c r="B14" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
-      <c r="I14" s="7"/>
-      <c r="J14" s="7"/>
-      <c r="K14" s="7"/>
-      <c r="L14" s="7"/>
-      <c r="M14" s="12">
-        <v>5</v>
-      </c>
-      <c r="N14" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="M14" s="9">
+        <v>5</v>
+      </c>
+      <c r="N14" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>5</v>
       </c>
-      <c r="B15" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
-      <c r="H15" s="7"/>
-      <c r="I15" s="7"/>
-      <c r="J15" s="7"/>
-      <c r="K15" s="7"/>
-      <c r="L15" s="7"/>
-      <c r="M15" s="12">
-        <v>5</v>
-      </c>
-      <c r="N15" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="M15" s="9">
+        <v>5</v>
+      </c>
+      <c r="N15" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>6</v>
       </c>
-      <c r="B16" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
-      <c r="H16" s="7"/>
-      <c r="I16" s="7"/>
-      <c r="J16" s="7"/>
-      <c r="K16" s="7"/>
-      <c r="L16" s="7"/>
-      <c r="M16" s="12">
-        <v>5</v>
-      </c>
-      <c r="N16" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="M16" s="9">
+        <v>5</v>
+      </c>
+      <c r="N16" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>7</v>
       </c>
-      <c r="B17" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
-      <c r="H17" s="7"/>
-      <c r="I17" s="7"/>
-      <c r="J17" s="7"/>
-      <c r="K17" s="7"/>
-      <c r="L17" s="7"/>
-      <c r="M17" s="12">
-        <v>5</v>
-      </c>
-      <c r="N17" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="M17" s="9">
+        <v>5</v>
+      </c>
+      <c r="N17" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>8</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="M18" s="13">
+      <c r="M18" s="9">
         <v>5</v>
       </c>
       <c r="N18" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>9</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="M19" s="13">
+      <c r="M19" s="9">
         <v>5</v>
       </c>
       <c r="N19" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>10</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="M20" s="13">
+      <c r="M20" s="9">
         <v>5</v>
       </c>
       <c r="N20" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>11</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="M21" s="13">
+      <c r="M21" s="9">
         <v>5</v>
       </c>
       <c r="N21" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>12</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="M22" s="13">
+      <c r="M22" s="9">
         <v>5</v>
       </c>
       <c r="N22" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>13</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="M23" s="13">
+      <c r="M23" s="9">
         <v>5</v>
       </c>
       <c r="N23" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>14</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="M24" s="13">
+      <c r="M24" s="9">
         <v>5</v>
       </c>
       <c r="N24" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>15</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="M25" s="13">
+      <c r="M25" s="9">
         <v>5</v>
       </c>
       <c r="N25" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>16</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="M26" s="13">
+      <c r="M26" s="9">
         <v>5</v>
       </c>
       <c r="N26" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="27" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>17</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="M27" s="13">
+      <c r="M27" s="9">
         <v>5</v>
       </c>
       <c r="N27" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="28" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>18</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="M28" s="13">
+      <c r="M28" s="9">
         <v>5</v>
       </c>
       <c r="N28" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="29" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>19</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="M29" s="13">
+      <c r="M29" s="9">
         <v>5</v>
       </c>
       <c r="N29" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="30" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>20</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="M30" s="13">
+      <c r="M30" s="9">
         <v>5</v>
       </c>
       <c r="N30" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="31" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>21</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="M31" s="13">
+      <c r="M31" s="9">
         <v>5</v>
       </c>
       <c r="N31" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="32" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
         <v>22</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="M32" s="13">
+      <c r="M32" s="9">
         <v>5</v>
       </c>
       <c r="N32" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
         <v>23</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="M33" s="13">
+      <c r="M33" s="9">
         <v>5</v>
       </c>
       <c r="N33" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="34" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
         <v>24</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="M34" s="13">
+      <c r="M34" s="9">
         <v>5</v>
       </c>
       <c r="N34" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="35" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
         <v>25</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="M35" s="13">
+      <c r="M35" s="9">
         <v>5</v>
       </c>
       <c r="N35" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B36" s="2"/>
     </row>
-    <row r="37" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B37" s="3" t="s">
         <v>10</v>
       </c>
       <c r="G37" s="5"/>
-      <c r="H37" s="11">
+      <c r="H37" s="8">
         <v>1</v>
       </c>
       <c r="K37" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="38" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B38" s="2"/>
     </row>
-    <row r="39" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="39" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="G6:H6"/>

</xml_diff>

<commit_message>
refactor: shared RequestForm component; request Excel template without gray fills
- Extract unified request form (25-item limit with counter, Enter-to-next-item focus, confirm dialog on submit) into components/orders/RequestForm.tsx; Requester/Warehouse/HeadOfSupply dashboards use it via props (showRequester, excelButton)
- Autocomplete: add optional focusKey prop to programmatically focus input
- REQUEST.xlsx: template re-uploaded without gray cell fills (spacer-row style fix removed)
</commit_message>
<xml_diff>
--- a/public/xls/REQUEST.xlsx
+++ b/public/xls/REQUEST.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stanislav/Desktop/PROJECTS/sv-progs-assistant/public/xls/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A210701-1BEF-E14D-9385-D20D9B99484A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47D1D684-3693-6A49-AE45-343AE882075D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15720" xr2:uid="{F3EB26A4-3A24-4C34-A589-8AC17AA75156}"/>
   </bookViews>
@@ -85,13 +85,6 @@
     </font>
     <font>
       <sz val="14"/>
-      <color rgb="FF507850"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <sz val="14"/>
       <color rgb="FF1A1A2E"/>
       <name val="Times New Roman"/>
       <family val="1"/>
@@ -120,19 +113,19 @@
       <family val="1"/>
       <charset val="204"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF8F9FA"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -158,25 +151,25 @@
   </cellStyleXfs>
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -495,509 +488,509 @@
   <dimension ref="A2:N39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="18" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="16384" width="9.1640625" style="1"/>
+    <col min="1" max="16384" width="9.1640625" style="2"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:14" ht="20" x14ac:dyDescent="0.2">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3" t="s">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
     </row>
     <row r="3" spans="1:14" ht="20" x14ac:dyDescent="0.2">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3" t="s">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-      <c r="L3" s="3"/>
-      <c r="M3" s="3"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:14" ht="20" x14ac:dyDescent="0.2">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="M4" s="3"/>
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
     </row>
     <row r="5" spans="1:14" ht="20" x14ac:dyDescent="0.2">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3" t="s">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
-      <c r="L5" s="3"/>
-      <c r="M5" s="3"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
     </row>
     <row r="6" spans="1:14" ht="20" x14ac:dyDescent="0.2">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3" t="s">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="10"/>
-      <c r="H6" s="10"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
-      <c r="L6" s="3"/>
-      <c r="M6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
     </row>
     <row r="7" spans="1:14" ht="20" x14ac:dyDescent="0.2">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
-      <c r="M7" s="3"/>
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
     </row>
     <row r="8" spans="1:14" ht="20" x14ac:dyDescent="0.2">
-      <c r="A8" s="3"/>
+      <c r="A8" s="1"/>
       <c r="B8" s="4"/>
-      <c r="C8" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="3"/>
-      <c r="M8" s="3"/>
+      <c r="C8" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
     </row>
     <row r="9" spans="1:14" ht="20" x14ac:dyDescent="0.2">
       <c r="A9" s="4"/>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
     </row>
     <row r="11" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>1</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="M11" s="9">
-        <v>5</v>
-      </c>
-      <c r="N11" s="1" t="s">
+      <c r="M11" s="6">
+        <v>5</v>
+      </c>
+      <c r="N11" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>2</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D12" s="7"/>
-      <c r="M12" s="9">
-        <v>5</v>
-      </c>
-      <c r="N12" s="1" t="s">
+      <c r="B12" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D12" s="8"/>
+      <c r="M12" s="6">
+        <v>5</v>
+      </c>
+      <c r="N12" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="1">
+      <c r="A13" s="2">
         <v>3</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="M13" s="9">
-        <v>5</v>
-      </c>
-      <c r="N13" s="1" t="s">
+      <c r="B13" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="M13" s="6">
+        <v>5</v>
+      </c>
+      <c r="N13" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="1">
-        <v>4</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="M14" s="9">
-        <v>5</v>
-      </c>
-      <c r="N14" s="1" t="s">
+      <c r="A14" s="2">
+        <v>4</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="M14" s="6">
+        <v>5</v>
+      </c>
+      <c r="N14" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="1">
-        <v>5</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="M15" s="9">
-        <v>5</v>
-      </c>
-      <c r="N15" s="1" t="s">
+      <c r="A15" s="2">
+        <v>5</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="M15" s="6">
+        <v>5</v>
+      </c>
+      <c r="N15" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>6</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="M16" s="9">
-        <v>5</v>
-      </c>
-      <c r="N16" s="1" t="s">
+      <c r="B16" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="M16" s="6">
+        <v>5</v>
+      </c>
+      <c r="N16" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="1">
+      <c r="A17" s="2">
         <v>7</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="M17" s="9">
-        <v>5</v>
-      </c>
-      <c r="N17" s="1" t="s">
+      <c r="B17" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="M17" s="6">
+        <v>5</v>
+      </c>
+      <c r="N17" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="18" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="1">
-        <v>8</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="M18" s="9">
-        <v>5</v>
-      </c>
-      <c r="N18" s="1" t="s">
+      <c r="A18" s="2">
+        <v>8</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="M18" s="6">
+        <v>5</v>
+      </c>
+      <c r="N18" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="19" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>9</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="M19" s="9">
-        <v>5</v>
-      </c>
-      <c r="N19" s="1" t="s">
+      <c r="B19" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="M19" s="6">
+        <v>5</v>
+      </c>
+      <c r="N19" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>10</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="M20" s="9">
-        <v>5</v>
-      </c>
-      <c r="N20" s="1" t="s">
+      <c r="B20" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="M20" s="6">
+        <v>5</v>
+      </c>
+      <c r="N20" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="21" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>11</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="M21" s="9">
-        <v>5</v>
-      </c>
-      <c r="N21" s="1" t="s">
+      <c r="B21" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="M21" s="6">
+        <v>5</v>
+      </c>
+      <c r="N21" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="22" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>12</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="M22" s="9">
-        <v>5</v>
-      </c>
-      <c r="N22" s="1" t="s">
+      <c r="B22" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="M22" s="6">
+        <v>5</v>
+      </c>
+      <c r="N22" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="23" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>13</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="M23" s="9">
-        <v>5</v>
-      </c>
-      <c r="N23" s="1" t="s">
+      <c r="B23" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="M23" s="6">
+        <v>5</v>
+      </c>
+      <c r="N23" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="24" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>14</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="M24" s="9">
-        <v>5</v>
-      </c>
-      <c r="N24" s="1" t="s">
+      <c r="B24" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="M24" s="6">
+        <v>5</v>
+      </c>
+      <c r="N24" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="25" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>15</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="M25" s="9">
-        <v>5</v>
-      </c>
-      <c r="N25" s="1" t="s">
+      <c r="B25" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="M25" s="6">
+        <v>5</v>
+      </c>
+      <c r="N25" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="26" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>16</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="M26" s="9">
-        <v>5</v>
-      </c>
-      <c r="N26" s="1" t="s">
+      <c r="B26" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="M26" s="6">
+        <v>5</v>
+      </c>
+      <c r="N26" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="27" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>17</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="M27" s="9">
-        <v>5</v>
-      </c>
-      <c r="N27" s="1" t="s">
+      <c r="B27" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="M27" s="6">
+        <v>5</v>
+      </c>
+      <c r="N27" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="28" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>18</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="M28" s="9">
-        <v>5</v>
-      </c>
-      <c r="N28" s="1" t="s">
+      <c r="B28" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="M28" s="6">
+        <v>5</v>
+      </c>
+      <c r="N28" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="29" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>19</v>
       </c>
-      <c r="B29" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="M29" s="9">
-        <v>5</v>
-      </c>
-      <c r="N29" s="1" t="s">
+      <c r="B29" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="M29" s="6">
+        <v>5</v>
+      </c>
+      <c r="N29" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="30" spans="1:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>20</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="M30" s="9">
-        <v>5</v>
-      </c>
-      <c r="N30" s="1" t="s">
+      <c r="B30" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="M30" s="6">
+        <v>5</v>
+      </c>
+      <c r="N30" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="31" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>21</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="M31" s="9">
-        <v>5</v>
-      </c>
-      <c r="N31" s="1" t="s">
+      <c r="B31" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="M31" s="6">
+        <v>5</v>
+      </c>
+      <c r="N31" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="32" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>22</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="M32" s="9">
-        <v>5</v>
-      </c>
-      <c r="N32" s="1" t="s">
+      <c r="B32" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="M32" s="6">
+        <v>5</v>
+      </c>
+      <c r="N32" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="33" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>23</v>
       </c>
-      <c r="B33" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="M33" s="9">
-        <v>5</v>
-      </c>
-      <c r="N33" s="1" t="s">
+      <c r="B33" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="M33" s="6">
+        <v>5</v>
+      </c>
+      <c r="N33" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="34" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>24</v>
       </c>
-      <c r="B34" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="M34" s="9">
-        <v>5</v>
-      </c>
-      <c r="N34" s="1" t="s">
+      <c r="B34" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="M34" s="6">
+        <v>5</v>
+      </c>
+      <c r="N34" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="35" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>25</v>
       </c>
-      <c r="B35" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="M35" s="9">
-        <v>5</v>
-      </c>
-      <c r="N35" s="1" t="s">
+      <c r="B35" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="M35" s="6">
+        <v>5</v>
+      </c>
+      <c r="N35" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="36" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B36" s="2"/>
+      <c r="B36" s="7"/>
     </row>
     <row r="37" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B37" s="3" t="s">
+      <c r="B37" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="G37" s="5"/>
-      <c r="H37" s="8">
+      <c r="G37" s="9"/>
+      <c r="H37" s="10">
         <v>1</v>
       </c>
-      <c r="K37" s="3" t="s">
+      <c r="K37" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="38" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B38" s="2"/>
+      <c r="B38" s="7"/>
     </row>
     <row r="39" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>

</xml_diff>